<commit_message>
Score each funded industry on the HKEX line that names it.
Board IPO totals stay as the denominator. Life and health, AI and robotics, and new energy now have their own following-year figures.

Co-authored-by: cheungyuenyuenhk <cheungyuenyuenhk@gmail.com>
</commit_message>
<xml_diff>
--- a/A1_CHEUNG_Yuk_Yuen/outputs/term_market.xlsx
+++ b/A1_CHEUNG_Yuk_Yuen/outputs/term_market.xlsx
@@ -11,8 +11,10 @@
     <sheet name="Inputs" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Year_after" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Chart_data" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Industry" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Industry!$A$1:$K$19</definedName>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Inputs!$A$1:$H$26</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -335,7 +337,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="145">
   <si>
     <t xml:space="preserve">year</t>
   </si>
@@ -590,6 +592,186 @@
   </si>
   <si>
     <t xml:space="preserve">ipo_funds_hkd_billion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">policy_industry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hkex_evidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">board_ipo_hkd_million</t>
+  </si>
+  <si>
+    <t xml:space="preserve">industry_share_of_ipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Life and health</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sichuan Kelun-Biotech Biopharmaceutical, ten largest IPOs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Market Statistics 2023, printed page 7. The printed name includes Biotech and the -B marker.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New energy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REPT BATTERO Energy, ten largest IPOs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Market Statistics 2023, printed page 7. The printed name includes Energy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sino-Synergy Hydrogen Energy Technology, ten largest IPOs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Market Statistics 2023, printed page 7. The printed name includes Hydrogen Energy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI and robotics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Horizon Robotics, ten largest IPOs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Market Statistics 2024, printed page 7. The 2023 address says AI and data science. The printed name says Robotics.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RoboSense Technology, ten largest IPOs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Market Statistics 2024, printed page 7.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Specialist technology</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chapter 18C listings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">not used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.hkex.com.hk/-/media/HKEX-Market/News/News-Release/2025/250227news/250227_FY-Results_e.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024 Final Results, p.11. First Chapter 18C listing was 13 June 2024. The five 18C industries are not split.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New economy, wider than the policy list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share of capital raised</t>
+  </si>
+  <si>
+    <t xml:space="preserve">almost 82%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024 Final Results, p.11. HKEX does not define new economy as the Policy Address industry list.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biotech Companies listed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.hkex.com.hk/-/media/HKEX-Market/Listing/How-We-Regulate/Listing-Committee/Listing-Committee-Report/AnnualRpt_2025dec.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Listing Committee Report 2025, p.3.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Specialist Technology Companies listed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Listing Committee Report 2025, p.3. Combined with the 16 biotech listings, HK$19.8 billion.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Life and health plus specialist technology</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Funds raised by the 16 biotech and 5 specialist technology listings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The page prints one combined sum. It is not split between the two chapters.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HengRui Pharma, H-share listing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Listing Committee Report 2025, p.2. Named separately from the HK$19.8 billion. Not added to it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contemporary Amperex Technology, named among the largest IPOs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Listing Committee Report 2025, p.2 names the company and does not print its proceeds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hesai, WeRide and Pony AI, named as homecoming listings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Listing Committee Report 2025, p.2. No separate proceeds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semi-conductors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No semiconductor IPO total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The 2024 address names semi-conductors and smart devices. The 2025 Listing Committee report does not.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Advanced materials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No advanced-materials IPO total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.hkex.com.hk/-/media/HKEX-Market/Listing/How-We-Regulate/Listing-Committee/Listing-Committee-Report/AnnualRpt_2023dec.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Advanced materials is one of five Chapter 18C industries, Listing Committee Report 2023, p.6. The 2025 count of five specialist technology listings is not split.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Film and creative industries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No film IPO line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Market Statistics 2024 does not report film or CreateSmart fundraising.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aerospace</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No aerospace IPO line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The highlights page has no industry split. Cirrus Aircraft, HK$1.51 billion, is on the 2024 ten-largest list, before this earmark.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Construction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No construction IPO line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The following year is not published.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share = this row's HK$ million / the board IPO total for the same window. Counts are not shares.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The 2025 denominator is HK$285,800 million, the Listing Committee's HK$285.8 billion, because 19.8 and 11.4 are printed there.</t>
   </si>
 </sst>
 </file>
@@ -722,7 +904,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -756,6 +938,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1099,11 +1285,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="41149632"/>
-        <c:axId val="36477487"/>
+        <c:axId val="35648728"/>
+        <c:axId val="64519664"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="41149632"/>
+        <c:axId val="35648728"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1135,7 +1321,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36477487"/>
+        <c:crossAx val="64519664"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1143,7 +1329,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="36477487"/>
+        <c:axId val="64519664"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1209,7 +1395,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="41149632"/>
+        <c:crossAx val="35648728"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1298,6 +1484,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2495,4 +2685,736 @@
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:K22"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="55"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <f aca="false">IF(F2="HK$ billion",E2*1000,IF(F2="HK$ million",E2,IF(F2="億元",E2*100,"")))</f>
+        <v>1560</v>
+      </c>
+      <c r="H2" s="9" t="n">
+        <v>46294.9</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <f aca="false">IF(OR(G2="",H2=""),"",G2/H2)</f>
+        <v>0.0336970163020117</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <f aca="false">IF(F3="HK$ billion",E3*1000,IF(F3="HK$ million",E3,IF(F3="億元",E3*100,"")))</f>
+        <v>2120</v>
+      </c>
+      <c r="H3" s="9" t="n">
+        <v>46294.9</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <f aca="false">IF(OR(G3="",H3=""),"",G3/H3)</f>
+        <v>0.0457933811283748</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <f aca="false">IF(F4="HK$ billion",E4*1000,IF(F4="HK$ million",E4,IF(F4="億元",E4*100,"")))</f>
+        <v>1560</v>
+      </c>
+      <c r="H4" s="9" t="n">
+        <v>46294.9</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <f aca="false">IF(OR(G4="",H4=""),"",G4/H4)</f>
+        <v>0.0336970163020117</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>6.09</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <f aca="false">IF(F5="HK$ billion",E5*1000,IF(F5="HK$ million",E5,IF(F5="億元",E5*100,"")))</f>
+        <v>6090</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>87477.8</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <f aca="false">IF(OR(G5="",H5=""),"",G5/H5)</f>
+        <v>0.06961766299564</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <f aca="false">IF(F6="HK$ billion",E6*1000,IF(F6="HK$ million",E6,IF(F6="億元",E6*100,"")))</f>
+        <v>1060</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>87477.8</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <f aca="false">IF(OR(G6="",H6=""),"",G6/H6)</f>
+        <v>0.0121173600616385</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="G7" s="3" t="str">
+        <f aca="false">IF(F7="HK$ billion",E7*1000,IF(F7="HK$ million",E7,IF(F7="億元",E7*100,"")))</f>
+        <v/>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F8" s="2"/>
+      <c r="G8" s="3" t="str">
+        <f aca="false">IF(F8="HK$ billion",E8*1000,IF(F8="HK$ million",E8,IF(F8="億元",E8*100,"")))</f>
+        <v/>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="G9" s="3" t="str">
+        <f aca="false">IF(F9="HK$ billion",E9*1000,IF(F9="HK$ million",E9,IF(F9="億元",E9*100,"")))</f>
+        <v/>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="G10" s="3" t="str">
+        <f aca="false">IF(F10="HK$ billion",E10*1000,IF(F10="HK$ million",E10,IF(F10="億元",E10*100,"")))</f>
+        <v/>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <f aca="false">IF(F11="HK$ billion",E11*1000,IF(F11="HK$ million",E11,IF(F11="億元",E11*100,"")))</f>
+        <v>19800</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>285800</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <f aca="false">IF(OR(G11="",H11=""),"",G11/H11)</f>
+        <v>0.0692792162351295</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <f aca="false">IF(F12="HK$ billion",E12*1000,IF(F12="HK$ million",E12,IF(F12="億元",E12*100,"")))</f>
+        <v>11400</v>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>285800</v>
+      </c>
+      <c r="I12" s="5" t="n">
+        <f aca="false">IF(OR(G12="",H12=""),"",G12/H12)</f>
+        <v>0.039888033589923</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G13" s="3" t="str">
+        <f aca="false">IF(F13="HK$ billion",E13*1000,IF(F13="HK$ million",E13,IF(F13="億元",E13*100,"")))</f>
+        <v/>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G14" s="3" t="str">
+        <f aca="false">IF(F14="HK$ billion",E14*1000,IF(F14="HK$ million",E14,IF(F14="億元",E14*100,"")))</f>
+        <v/>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G15" s="3" t="str">
+        <f aca="false">IF(F15="HK$ billion",E15*1000,IF(F15="HK$ million",E15,IF(F15="億元",E15*100,"")))</f>
+        <v/>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G16" s="3" t="str">
+        <f aca="false">IF(F16="HK$ billion",E16*1000,IF(F16="HK$ million",E16,IF(F16="億元",E16*100,"")))</f>
+        <v/>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G17" s="3" t="str">
+        <f aca="false">IF(F17="HK$ billion",E17*1000,IF(F17="HK$ million",E17,IF(F17="億元",E17*100,"")))</f>
+        <v/>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G18" s="3" t="str">
+        <f aca="false">IF(F18="HK$ billion",E18*1000,IF(F18="HK$ million",E18,IF(F18="億元",E18*100,"")))</f>
+        <v/>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G19" s="3" t="str">
+        <f aca="false">IF(F19="HK$ billion",E19*1000,IF(F19="HK$ million",E19,IF(F19="億元",E19*100,"")))</f>
+        <v/>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="s">
+        <v>144</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K19"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Compare Chapter 18C listings with the market from the rule's effective date.
The count starts at zero on 31 March 2023. Base Rate and Southbound turnover sit beside the later listings, and the Industry-Oriented Fund stays out because it has no disbursement date.

Co-authored-by: cheungyuenyuenhk <cheungyuenyuenhk@gmail.com>
</commit_message>
<xml_diff>
--- a/A1_CHEUNG_Yuk_Yuen/outputs/term_market.xlsx
+++ b/A1_CHEUNG_Yuk_Yuen/outputs/term_market.xlsx
@@ -12,6 +12,8 @@
     <sheet name="Year_after" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Chart_data" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Industry" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="C18_listings" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="C18_before_after" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Industry!$A$1:$K$19</definedName>
@@ -337,7 +339,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="192">
   <si>
     <t xml:space="preserve">year</t>
   </si>
@@ -772,18 +774,160 @@
   </si>
   <si>
     <t xml:space="preserve">The 2025 denominator is HK$285,800 million, the Listing Committee's HK$285.8 billion, because 19.8 and 11.4 are printed there.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">company</t>
+  </si>
+  <si>
+    <t xml:space="preserve">listing_date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">funds_hkd_million</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XtalPi Holdings Ltd.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024-06-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.hkexgroup.com/Media-Centre/Insight/Insight/2026/HKEX-Insight/18C-Explained?sc_lang=en</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Black Sesame International Holdings Ltd.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024-08-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shenzhen Dobot Corp. Ltd.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024-12-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beijing Yunji Technology Co., Ltd.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-10-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deepexi Technology Co., Ltd.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-10-28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WeRide Inc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-11-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CiDi Inc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-12-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beijing 51World Digital Twin Technology Co., Ltd.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-12-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shanghai Biren Technology Co., Ltd.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-01-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Knowledge Atlas Technology JSC Ltd.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-01-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MiniMax Group Inc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-01-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guangdong Huayan Robotics Co., Ltd.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shandong Extreme Vision Technology Co., Ltd.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shanghai FourSemi Semiconductor Co., Ltd.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page total, HK$ billion, as printed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sum of the rows, HK$ million</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c18_listings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c18_funds_hkd_million</t>
+  </si>
+  <si>
+    <t xml:space="preserve">base_rate_year_end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">southbound_adt_hkd_billion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c18_share_of_board_ipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Before Chapter 18C. Base Rate end-2022. Southbound ADT. IPO from Market Statistics 2022.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chapter effective 31 Mar 2023. No 18C listing this year. Base Rate end-2023 was 5.75%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Three 18C listings. Base Rate cut from 5.75% to 4.75%. Southbound ADT HK$48.2 billion.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Five 18C listings. Base Rate cut from 4.75% to 4.00%. Southbound ADT HK$121.1 billion. Board IPO is the Listing Committee figure.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Listings through 31 Mar 2026 only. A full-year Base Rate, Southbound ADT and board IPO are not stated in source.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chapter 18C effective 31 March 2023. First listing 13 June 2024.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The I&amp;T Industry-Oriented Fund has no disbursement date in the 2026 Policy Address. It is not in this table.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2022 Base Rate: HKMA Annual Report 2022. 2023 and 2024: HKMA Annual Report 2024. 2025: HKMA Annual Report 2025.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Southbound ADT: HKEX Stock Connect 2025 Review, February 2026.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
     <numFmt numFmtId="168" formatCode="#,##0"/>
+    <numFmt numFmtId="169" formatCode="0.00%"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -904,7 +1048,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -942,6 +1086,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1285,11 +1441,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="35648728"/>
-        <c:axId val="64519664"/>
+        <c:axId val="9867641"/>
+        <c:axId val="92096495"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="35648728"/>
+        <c:axId val="9867641"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1321,7 +1477,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="64519664"/>
+        <c:crossAx val="92096495"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1329,7 +1485,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="64519664"/>
+        <c:axId val="92096495"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1395,7 +1551,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="35648728"/>
+        <c:crossAx val="9867641"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3417,4 +3573,521 @@
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E18"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="55"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D2" s="10" t="n">
+        <v>1036</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D3" s="10" t="n">
+        <v>1036</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>759</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>710</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>2392</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>1422</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D9" s="10" t="n">
+        <v>731</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>6420</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>5540</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D13" s="10" t="n">
+        <v>1579</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>499</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>480</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>28.4</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="B18" s="11" t="n">
+        <f aca="false">SUM(D2:D15)</f>
+        <v>28435</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="78"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B2" s="7" t="n">
+        <f aca="false">COUNTIF(C18_listings!C:C,A2)</f>
+        <v>0</v>
+      </c>
+      <c r="C2" s="11" t="n">
+        <f aca="false">SUMIF(C18_listings!C:C,A2,C18_listings!D:D)</f>
+        <v>0</v>
+      </c>
+      <c r="D2" s="12" t="n">
+        <v>0.0475</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="F2" s="9" t="n">
+        <v>104570.3</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <f aca="false">IF(F2="", "", C2/F2)</f>
+        <v>0</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B3" s="7" t="n">
+        <f aca="false">COUNTIF(C18_listings!C:C,A3)</f>
+        <v>0</v>
+      </c>
+      <c r="C3" s="11" t="n">
+        <f aca="false">SUMIF(C18_listings!C:C,A3,C18_listings!D:D)</f>
+        <v>0</v>
+      </c>
+      <c r="D3" s="12" t="n">
+        <v>0.0575</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>46294.9</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <f aca="false">IF(F3="", "", C3/F3)</f>
+        <v>0</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B4" s="7" t="n">
+        <f aca="false">COUNTIF(C18_listings!C:C,A4)</f>
+        <v>3</v>
+      </c>
+      <c r="C4" s="11" t="n">
+        <f aca="false">SUMIF(C18_listings!C:C,A4,C18_listings!D:D)</f>
+        <v>2903</v>
+      </c>
+      <c r="D4" s="12" t="n">
+        <v>0.0475</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>87477.8</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <f aca="false">IF(F4="", "", C4/F4)</f>
+        <v>0.0331855625084307</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <f aca="false">COUNTIF(C18_listings!C:C,A5)</f>
+        <v>5</v>
+      </c>
+      <c r="C5" s="11" t="n">
+        <f aca="false">SUMIF(C18_listings!C:C,A5,C18_listings!D:D)</f>
+        <v>6014</v>
+      </c>
+      <c r="D5" s="12" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>121.1</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>285800</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <f aca="false">IF(F5="", "", C5/F5)</f>
+        <v>0.0210426871938418</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B6" s="7" t="n">
+        <f aca="false">COUNTIF(C18_listings!C:C,A6)</f>
+        <v>6</v>
+      </c>
+      <c r="C6" s="11" t="n">
+        <f aca="false">SUMIF(C18_listings!C:C,A6,C18_listings!D:D)</f>
+        <v>19518</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>191</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fit the submission files to the Lecture 3 handout.
- One-page report.pdf with step timeline, four concepts, result paths, key chart and self-assessment; full tables move to outputs/analysis.pdf.
- Drop the unsupported Plan Mode claim; describe what the agent did instead of first-person 'I read'.
- Skill note cut to eight lines with what worked, what failed and what changed.
- skill_intro gains install command and invocation; reflection follows the handout sections, including work fit, and states how the trial draft was made.

Co-authored-by: cheungyuenyuenhk <cheungyuenyuenhk@gmail.com>
</commit_message>
<xml_diff>
--- a/A1_CHEUNG_Yuk_Yuen/outputs/term_market.xlsx
+++ b/A1_CHEUNG_Yuk_Yuen/outputs/term_market.xlsx
@@ -5677,11 +5677,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="80236774"/>
-        <c:axId val="15274151"/>
+        <c:axId val="2995849"/>
+        <c:axId val="80425859"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="80236774"/>
+        <c:axId val="2995849"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5747,7 +5747,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="15274151"/>
+        <c:crossAx val="80425859"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5755,7 +5755,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="15274151"/>
+        <c:axId val="80425859"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5821,7 +5821,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80236774"/>
+        <c:crossAx val="2995849"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>